<commit_message>
pending line and checkout validations
</commit_message>
<xml_diff>
--- a/docs/official/EInvoice_Data_Dictionary.xlsx
+++ b/docs/official/EInvoice_Data_Dictionary.xlsx
@@ -2982,7 +2982,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3051,6 +3051,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor theme="5" tint="0.59999389629810485"/>
       </patternFill>
     </fill>
   </fills>
@@ -3350,7 +3356,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -3660,6 +3666,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="18" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="13" borderId="16" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -17297,7 +17309,7 @@
       </c>
     </row>
     <row r="85" ht="50.149999999999999" customHeight="1">
-      <c r="A85" s="97" t="s">
+      <c r="A85" s="111" t="s">
         <v>586</v>
       </c>
       <c r="B85" s="60" t="s">
@@ -17365,7 +17377,7 @@
       </c>
     </row>
     <row r="86" ht="50.149999999999999" customHeight="1">
-      <c r="A86" s="97" t="s">
+      <c r="A86" s="111" t="s">
         <v>595</v>
       </c>
       <c r="B86" s="60" t="s">
@@ -17437,7 +17449,7 @@
       </c>
     </row>
     <row r="87" ht="50.149999999999999" customHeight="1">
-      <c r="A87" s="97" t="s">
+      <c r="A87" s="111" t="s">
         <v>604</v>
       </c>
       <c r="B87" s="60" t="s">
@@ -17503,7 +17515,7 @@
       </c>
     </row>
     <row r="88" ht="46.5">
-      <c r="A88" s="97" t="s">
+      <c r="A88" s="111" t="s">
         <v>609</v>
       </c>
       <c r="B88" s="60" t="s">
@@ -17535,7 +17547,7 @@
       <c r="L88" s="60" t="s">
         <v>615</v>
       </c>
-      <c r="M88" s="60" t="s">
+      <c r="M88" s="112" t="s">
         <v>616</v>
       </c>
       <c r="N88" s="67"/>
@@ -17575,7 +17587,7 @@
       </c>
     </row>
     <row r="89" ht="50.149999999999999" customHeight="1">
-      <c r="A89" s="97" t="s">
+      <c r="A89" s="111" t="s">
         <v>618</v>
       </c>
       <c r="B89" s="60" t="s">
@@ -17645,7 +17657,7 @@
       </c>
     </row>
     <row r="90" ht="50.149999999999999" customHeight="1">
-      <c r="A90" s="97" t="s">
+      <c r="A90" s="111" t="s">
         <v>620</v>
       </c>
       <c r="B90" s="60" t="s">
@@ -17697,7 +17709,7 @@
       <c r="T90" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="U90" s="111"/>
+      <c r="U90" s="113"/>
       <c r="V90" s="60" t="s">
         <v>69</v>
       </c>
@@ -17713,7 +17725,7 @@
       </c>
     </row>
     <row r="91" ht="68.5" customHeight="1">
-      <c r="A91" s="97" t="s">
+      <c r="A91" s="111" t="s">
         <v>624</v>
       </c>
       <c r="B91" s="60" t="s">
@@ -18189,7 +18201,7 @@
       <c r="T97" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="U97" s="112"/>
+      <c r="U97" s="114"/>
       <c r="V97" s="60" t="s">
         <v>81</v>
       </c>
@@ -19151,7 +19163,7 @@
       <c r="T111" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="U111" s="111"/>
+      <c r="U111" s="113"/>
       <c r="V111" s="60" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
parties validation and xml formating done, better renaming
</commit_message>
<xml_diff>
--- a/docs/official/EInvoice_Data_Dictionary.xlsx
+++ b/docs/official/EInvoice_Data_Dictionary.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="748">
   <si>
     <t xml:space="preserve">Zakat, Tax and Customs Authority (ZATCA)</t>
   </si>
@@ -1309,6 +1309,9 @@
   <si>
     <t xml:space="preserve">BR-KSA-14
 BR-KSA-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation moved to lines</t>
   </si>
   <si>
     <t xml:space="preserve">Buyer address line 1 - the main address line in an address</t>
@@ -3356,7 +3359,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="114">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -3669,9 +3672,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="13" borderId="16" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -12844,7 +12844,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="21" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="21" ht="50.149999999999999" customHeight="1">
       <c r="A21" s="93" t="s">
         <v>212</v>
       </c>
@@ -12914,7 +12914,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="22" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="22" ht="50.149999999999999" customHeight="1">
       <c r="A22" s="97" t="s">
         <v>223</v>
       </c>
@@ -12984,7 +12984,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="23" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="23" ht="50.149999999999999" customHeight="1">
       <c r="A23" s="60" t="s">
         <v>232</v>
       </c>
@@ -13050,7 +13050,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="24" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="24" ht="50.149999999999999" customHeight="1">
       <c r="A24" s="60" t="s">
         <v>236</v>
       </c>
@@ -13118,7 +13118,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="25" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="25" ht="50.149999999999999" customHeight="1">
       <c r="A25" s="97" t="s">
         <v>241</v>
       </c>
@@ -13188,7 +13188,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="26" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="26" ht="50.149999999999999" customHeight="1">
       <c r="A26" s="60" t="s">
         <v>247</v>
       </c>
@@ -13258,7 +13258,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="27" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="27" ht="50.149999999999999" customHeight="1">
       <c r="A27" s="97" t="s">
         <v>252</v>
       </c>
@@ -13330,7 +13330,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="28" s="99" customFormat="1" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="28" s="99" customFormat="1" ht="50.149999999999999" customHeight="1">
       <c r="A28" s="97" t="s">
         <v>259</v>
       </c>
@@ -13398,7 +13398,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="29" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="29" ht="50.149999999999999" customHeight="1">
       <c r="A29" s="61" t="s">
         <v>264</v>
       </c>
@@ -13468,7 +13468,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="30" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="30" ht="50.149999999999999" customHeight="1">
       <c r="A30" s="60" t="s">
         <v>269</v>
       </c>
@@ -13538,7 +13538,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="31" ht="129" hidden="1" customHeight="1">
+    <row r="31" ht="129" customHeight="1">
       <c r="A31" s="100" t="s">
         <v>275</v>
       </c>
@@ -13608,7 +13608,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="32" ht="50" hidden="1" customHeight="1">
+    <row r="32" ht="50" customHeight="1">
       <c r="A32" s="60" t="s">
         <v>283</v>
       </c>
@@ -13676,7 +13676,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="33" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="33" ht="50.149999999999999" customHeight="1">
       <c r="A33" s="97" t="s">
         <v>289</v>
       </c>
@@ -13745,29 +13745,32 @@
       <c r="Z33" s="60" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="34" ht="50.149999999999999" hidden="1" customHeight="1">
+      <c r="AA33" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="34" ht="50.149999999999999" customHeight="1">
       <c r="A34" s="97" t="s">
         <v>223</v>
       </c>
       <c r="B34" s="60" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C34" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D34" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E34" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F34" s="60" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G34" s="67"/>
       <c r="H34" s="60" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="I34" s="60" t="s">
         <v>65</v>
@@ -13777,10 +13780,10 @@
       </c>
       <c r="K34" s="67"/>
       <c r="L34" s="60" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M34" s="60" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N34" s="67"/>
       <c r="O34" s="60" t="s">
@@ -13816,28 +13819,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="35" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="35" ht="50.149999999999999" customHeight="1">
       <c r="A35" s="97" t="s">
         <v>232</v>
       </c>
       <c r="B35" s="60" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C35" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D35" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E35" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F35" s="60" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G35" s="67"/>
       <c r="H35" s="60" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="I35" s="60" t="s">
         <v>65</v>
@@ -13876,34 +13879,34 @@
       </c>
       <c r="X35" s="67"/>
       <c r="Y35" s="65" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="Z35" s="60" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="36" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="36" ht="50.149999999999999" customHeight="1">
       <c r="A36" s="97" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B36" s="60" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C36" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D36" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E36" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F36" s="60" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G36" s="67"/>
       <c r="H36" s="60" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I36" s="60" t="s">
         <v>65</v>
@@ -13913,10 +13916,10 @@
       </c>
       <c r="K36" s="67"/>
       <c r="L36" s="60" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M36" s="60" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N36" s="67"/>
       <c r="O36" s="60" t="s">
@@ -13950,28 +13953,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="37" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="37" ht="50.149999999999999" customHeight="1">
       <c r="A37" s="97" t="s">
         <v>241</v>
       </c>
       <c r="B37" s="60" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C37" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D37" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E37" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F37" s="60" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G37" s="67"/>
       <c r="H37" s="60" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I37" s="60" t="s">
         <v>65</v>
@@ -13982,7 +13985,7 @@
       <c r="K37" s="67"/>
       <c r="L37" s="60"/>
       <c r="M37" s="60" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="N37" s="67"/>
       <c r="O37" s="60" t="s">
@@ -14016,28 +14019,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="38" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="38" ht="50.149999999999999" customHeight="1">
       <c r="A38" s="97" t="s">
         <v>247</v>
       </c>
       <c r="B38" s="60" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C38" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D38" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E38" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F38" s="60" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G38" s="67"/>
       <c r="H38" s="60" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I38" s="60" t="s">
         <v>65</v>
@@ -14047,10 +14050,10 @@
       </c>
       <c r="K38" s="67"/>
       <c r="L38" s="60" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M38" s="60" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N38" s="67"/>
       <c r="O38" s="60" t="s">
@@ -14086,28 +14089,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="39" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="39" ht="50.149999999999999" customHeight="1">
       <c r="A39" s="97" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B39" s="60" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C39" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D39" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E39" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F39" s="60" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G39" s="67"/>
       <c r="H39" s="60" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="I39" s="60" t="s">
         <v>65</v>
@@ -14117,10 +14120,10 @@
       </c>
       <c r="K39" s="67"/>
       <c r="L39" s="60" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M39" s="60" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="N39" s="67"/>
       <c r="O39" s="60" t="s">
@@ -14154,28 +14157,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="40" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="40" ht="50.149999999999999" customHeight="1">
       <c r="A40" s="97" t="s">
         <v>259</v>
       </c>
       <c r="B40" s="60" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C40" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D40" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E40" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F40" s="60" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G40" s="67"/>
       <c r="H40" s="60" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="I40" s="60" t="s">
         <v>65</v>
@@ -14220,28 +14223,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="41" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="41" ht="50.149999999999999" customHeight="1">
       <c r="A41" s="97" t="s">
         <v>264</v>
       </c>
       <c r="B41" s="60" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C41" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D41" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E41" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F41" s="60" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G41" s="67"/>
       <c r="H41" s="60" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="I41" s="60" t="s">
         <v>65</v>
@@ -14252,7 +14255,7 @@
       <c r="K41" s="67"/>
       <c r="L41" s="60"/>
       <c r="M41" s="60" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="N41" s="67"/>
       <c r="O41" s="60" t="s">
@@ -14282,34 +14285,34 @@
       </c>
       <c r="X41" s="67"/>
       <c r="Y41" s="65" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="Z41" s="60" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="42" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="42" ht="50.149999999999999" customHeight="1">
       <c r="A42" s="97" t="s">
         <v>269</v>
       </c>
       <c r="B42" s="60" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C42" s="66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D42" s="63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E42" s="63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F42" s="60" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G42" s="67"/>
       <c r="H42" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I42" s="60" t="s">
         <v>165</v>
@@ -14319,10 +14322,10 @@
       </c>
       <c r="K42" s="67"/>
       <c r="L42" s="60" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M42" s="60" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N42" s="67"/>
       <c r="O42" s="60" t="s">
@@ -14358,15 +14361,15 @@
         <v>222</v>
       </c>
     </row>
-    <row r="43" ht="105" hidden="1">
+    <row r="43" ht="105">
       <c r="A43" s="102" t="s">
         <v>275</v>
       </c>
       <c r="B43" s="60" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C43" s="62" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D43" s="63" t="s">
         <v>292</v>
@@ -14375,11 +14378,11 @@
         <v>293</v>
       </c>
       <c r="F43" s="60" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G43" s="67"/>
       <c r="H43" s="60" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I43" s="60" t="s">
         <v>165</v>
@@ -14390,7 +14393,7 @@
       <c r="K43" s="67"/>
       <c r="L43" s="61"/>
       <c r="M43" s="61" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="N43" s="67"/>
       <c r="O43" s="60" t="s">
@@ -14420,21 +14423,21 @@
       </c>
       <c r="X43" s="67"/>
       <c r="Y43" s="98" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Z43" s="60" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="44" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="44" ht="50.149999999999999" customHeight="1">
       <c r="A44" s="97" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B44" s="60" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C44" s="66" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D44" s="63" t="s">
         <v>292</v>
@@ -14443,11 +14446,11 @@
         <v>293</v>
       </c>
       <c r="F44" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G44" s="67"/>
       <c r="H44" s="60" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I44" s="60" t="s">
         <v>165</v>
@@ -14458,7 +14461,7 @@
       <c r="K44" s="67"/>
       <c r="L44" s="60"/>
       <c r="M44" s="61" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="N44" s="67"/>
       <c r="O44" s="60" t="s">
@@ -14488,7 +14491,7 @@
       </c>
       <c r="X44" s="67"/>
       <c r="Y44" s="65" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="Z44" s="60" t="s">
         <v>222</v>
@@ -14496,26 +14499,26 @@
     </row>
     <row r="45" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A45" s="97" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B45" s="60" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C45" s="66" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D45" s="63" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E45" s="63" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F45" s="60" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G45" s="67"/>
       <c r="H45" s="60" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I45" s="60" t="s">
         <v>65</v>
@@ -14526,7 +14529,7 @@
       <c r="K45" s="67"/>
       <c r="L45" s="60"/>
       <c r="M45" s="61" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="N45" s="67"/>
       <c r="O45" s="103" t="s">
@@ -14556,7 +14559,7 @@
       </c>
       <c r="X45" s="67"/>
       <c r="Y45" s="65" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Z45" s="60" t="s">
         <v>83</v>
@@ -14564,26 +14567,26 @@
     </row>
     <row r="46" ht="67.5" hidden="1" customHeight="1">
       <c r="A46" s="60" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B46" s="60" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C46" s="66" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D46" s="63" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E46" s="63" t="s">
         <v>75</v>
       </c>
       <c r="F46" s="60" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G46" s="67"/>
       <c r="H46" s="60" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I46" s="60" t="s">
         <v>65</v>
@@ -14594,7 +14597,7 @@
       <c r="K46" s="67"/>
       <c r="L46" s="60"/>
       <c r="M46" s="61" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="N46" s="67"/>
       <c r="O46" s="103" t="s">
@@ -14624,7 +14627,7 @@
       </c>
       <c r="X46" s="67"/>
       <c r="Y46" s="65" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Z46" s="60" t="s">
         <v>83</v>
@@ -14632,26 +14635,26 @@
     </row>
     <row r="47" ht="45" hidden="1">
       <c r="A47" s="60" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B47" s="71" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C47" s="60" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D47" s="104" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E47" s="70" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F47" s="60" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G47" s="67"/>
       <c r="H47" s="60" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I47" s="60" t="s">
         <v>78</v>
@@ -14661,10 +14664,10 @@
       </c>
       <c r="K47" s="67"/>
       <c r="L47" s="60" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M47" s="60" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="N47" s="67"/>
       <c r="O47" s="60" t="s">
@@ -14686,7 +14689,7 @@
         <v>141</v>
       </c>
       <c r="U47" s="60" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="V47" s="60" t="s">
         <v>69</v>
@@ -14696,34 +14699,34 @@
       </c>
       <c r="X47" s="67"/>
       <c r="Y47" s="65" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="Z47" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="48" ht="165" hidden="1">
       <c r="A48" s="97" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B48" s="105" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C48" s="60" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D48" s="106" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E48" s="73" t="s">
         <v>75</v>
       </c>
       <c r="F48" s="60" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G48" s="67"/>
       <c r="H48" s="60" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I48" s="60" t="s">
         <v>140</v>
@@ -14734,7 +14737,7 @@
       <c r="K48" s="67"/>
       <c r="L48" s="60"/>
       <c r="M48" s="60" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="N48" s="67"/>
       <c r="O48" s="60" t="s">
@@ -14756,7 +14759,7 @@
         <v>68</v>
       </c>
       <c r="U48" s="60" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="V48" s="60" t="s">
         <v>69</v>
@@ -14766,7 +14769,7 @@
       </c>
       <c r="X48" s="67"/>
       <c r="Y48" s="107" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="Z48" s="60" t="s">
         <v>83</v>
@@ -14774,26 +14777,26 @@
     </row>
     <row r="49" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A49" s="60" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B49" s="71" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C49" s="60" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D49" s="108" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E49" s="70" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F49" s="97" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G49" s="67"/>
       <c r="H49" s="60" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="I49" s="60" t="s">
         <v>65</v>
@@ -14832,34 +14835,34 @@
       </c>
       <c r="X49" s="67"/>
       <c r="Y49" s="65" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="Z49" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="50" ht="30" hidden="1">
       <c r="A50" s="61" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B50" s="105" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C50" s="61" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D50" s="61" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E50" s="61" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F50" s="102" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G50" s="64"/>
       <c r="H50" s="61" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I50" s="61" t="s">
         <v>65</v>
@@ -14869,7 +14872,7 @@
       </c>
       <c r="K50" s="64"/>
       <c r="L50" s="61" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="M50" s="61"/>
       <c r="N50" s="64"/>
@@ -14900,45 +14903,45 @@
       </c>
       <c r="X50" s="64"/>
       <c r="Y50" s="107" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="Z50" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="51" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A51" s="60" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B51" s="71" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C51" s="60" t="s">
         <v>60</v>
       </c>
       <c r="D51" s="104" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E51" s="109" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F51" s="60" t="s">
         <v>106</v>
       </c>
       <c r="G51" s="67"/>
       <c r="H51" s="60" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="I51" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J51" s="60" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K51" s="67"/>
       <c r="L51" s="60"/>
       <c r="M51" s="60" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="N51" s="67"/>
       <c r="O51" s="60" t="s">
@@ -14968,45 +14971,45 @@
       </c>
       <c r="X51" s="67"/>
       <c r="Y51" s="65" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="Z51" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="52" ht="60" hidden="1">
       <c r="A52" s="60" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B52" s="60" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C52" s="110" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D52" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E52" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F52" s="60" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G52" s="67"/>
       <c r="H52" s="60" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="I52" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J52" s="60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K52" s="67"/>
       <c r="L52" s="60"/>
       <c r="M52" s="61" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="N52" s="67"/>
       <c r="O52" s="60" t="s">
@@ -15028,7 +15031,7 @@
         <v>17</v>
       </c>
       <c r="U52" s="60" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="V52" s="60" t="s">
         <v>69</v>
@@ -15038,47 +15041,47 @@
       </c>
       <c r="X52" s="67"/>
       <c r="Y52" s="65" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="Z52" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="53" ht="45" hidden="1">
       <c r="A53" s="60" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B53" s="60" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C53" s="69" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D53" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E53" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F53" s="60" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G53" s="67"/>
       <c r="H53" s="60" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="I53" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J53" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K53" s="67"/>
       <c r="L53" s="60" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="M53" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N53" s="67"/>
       <c r="O53" s="60" t="s">
@@ -15100,7 +15103,7 @@
         <v>17</v>
       </c>
       <c r="U53" s="60" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="V53" s="60" t="s">
         <v>81</v>
@@ -15110,34 +15113,34 @@
       </c>
       <c r="X53" s="67"/>
       <c r="Y53" s="65" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Z53" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="54" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A54" s="60" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B54" s="60" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C54" s="69" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D54" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E54" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F54" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G54" s="67"/>
       <c r="H54" s="60" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I54" s="60" t="s">
         <v>165</v>
@@ -15147,7 +15150,7 @@
       </c>
       <c r="K54" s="67"/>
       <c r="L54" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M54" s="61" t="s">
         <v>150</v>
@@ -15183,44 +15186,44 @@
         <v>151</v>
       </c>
       <c r="Z54" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="55" ht="60" hidden="1">
       <c r="A55" s="60" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B55" s="60" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C55" s="69" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D55" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E55" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F55" s="60" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G55" s="67"/>
       <c r="H55" s="60" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="I55" s="60" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="J55" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K55" s="67"/>
       <c r="L55" s="60" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="M55" s="61" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="N55" s="67"/>
       <c r="O55" s="60" t="s">
@@ -15242,7 +15245,7 @@
         <v>17</v>
       </c>
       <c r="U55" s="60" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="V55" s="60" t="s">
         <v>69</v>
@@ -15252,34 +15255,34 @@
       </c>
       <c r="X55" s="67"/>
       <c r="Y55" s="65" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="Z55" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="56" ht="45" hidden="1">
       <c r="A56" s="60" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B56" s="60" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C56" s="69" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D56" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E56" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F56" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G56" s="67"/>
       <c r="H56" s="60" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="I56" s="60" t="s">
         <v>165</v>
@@ -15289,7 +15292,7 @@
       </c>
       <c r="K56" s="67"/>
       <c r="L56" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M56" s="60" t="s">
         <v>150</v>
@@ -15325,31 +15328,31 @@
         <v>151</v>
       </c>
       <c r="Z56" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="57" ht="75" hidden="1">
       <c r="A57" s="60" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B57" s="60" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C57" s="69" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D57" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E57" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F57" s="60" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G57" s="67"/>
       <c r="H57" s="60" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="I57" s="60" t="s">
         <v>165</v>
@@ -15359,10 +15362,10 @@
       </c>
       <c r="K57" s="67"/>
       <c r="L57" s="60" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="M57" s="60" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N57" s="67"/>
       <c r="O57" s="60" t="s">
@@ -15384,7 +15387,7 @@
         <v>17</v>
       </c>
       <c r="U57" s="60" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="V57" s="60" t="s">
         <v>69</v>
@@ -15394,47 +15397,47 @@
       </c>
       <c r="X57" s="67"/>
       <c r="Y57" s="65" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="Z57" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="58" ht="75" hidden="1">
       <c r="A58" s="60" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B58" s="60" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C58" s="69" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D58" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E58" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F58" s="60" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G58" s="67"/>
       <c r="H58" s="60" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I58" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J58" s="60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K58" s="67"/>
       <c r="L58" s="60" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="M58" s="60" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="N58" s="67"/>
       <c r="O58" s="60" t="s">
@@ -15456,7 +15459,7 @@
         <v>17</v>
       </c>
       <c r="U58" s="60" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="V58" s="60" t="s">
         <v>69</v>
@@ -15466,45 +15469,45 @@
       </c>
       <c r="X58" s="67"/>
       <c r="Y58" s="65" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="Z58" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="59" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A59" s="60" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B59" s="60" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C59" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D59" s="73" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E59" s="73" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F59" s="60" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G59" s="67"/>
       <c r="H59" s="60" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="I59" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J59" s="60" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K59" s="67"/>
       <c r="L59" s="60"/>
       <c r="M59" s="60" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="N59" s="67"/>
       <c r="O59" s="60" t="s">
@@ -15534,47 +15537,47 @@
       </c>
       <c r="X59" s="67"/>
       <c r="Y59" s="65" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="Z59" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="60" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A60" s="60" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B60" s="60" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C60" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D60" s="73" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E60" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F60" s="60" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G60" s="67"/>
       <c r="H60" s="60" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="I60" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J60" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K60" s="67"/>
       <c r="L60" s="60" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="M60" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N60" s="67"/>
       <c r="O60" s="60" t="s">
@@ -15596,7 +15599,7 @@
         <v>68</v>
       </c>
       <c r="U60" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V60" s="60" t="s">
         <v>69</v>
@@ -15606,34 +15609,34 @@
       </c>
       <c r="X60" s="67"/>
       <c r="Y60" s="65" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="Z60" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="61" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A61" s="60" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B61" s="60" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C61" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D61" s="73" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E61" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F61" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G61" s="67"/>
       <c r="H61" s="60" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="I61" s="60" t="s">
         <v>78</v>
@@ -15643,7 +15646,7 @@
       </c>
       <c r="K61" s="67"/>
       <c r="L61" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M61" s="60" t="s">
         <v>150</v>
@@ -15679,44 +15682,44 @@
         <v>151</v>
       </c>
       <c r="Z61" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="62" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A62" s="60" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B62" s="60" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C62" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D62" s="73" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E62" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F62" s="60" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G62" s="67"/>
       <c r="H62" s="60" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I62" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J62" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K62" s="67"/>
       <c r="L62" s="60" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M62" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N62" s="67"/>
       <c r="O62" s="60" t="s">
@@ -15738,7 +15741,7 @@
         <v>17</v>
       </c>
       <c r="U62" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V62" s="61" t="s">
         <v>69</v>
@@ -15748,34 +15751,34 @@
       </c>
       <c r="X62" s="67"/>
       <c r="Y62" s="65" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="Z62" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="63" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A63" s="60" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B63" s="60" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C63" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D63" s="73" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E63" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F63" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G63" s="67"/>
       <c r="H63" s="60" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="I63" s="60" t="s">
         <v>165</v>
@@ -15785,7 +15788,7 @@
       </c>
       <c r="K63" s="67"/>
       <c r="L63" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M63" s="60" t="s">
         <v>150</v>
@@ -15821,44 +15824,44 @@
         <v>151</v>
       </c>
       <c r="Z63" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="64" ht="99" hidden="1" customHeight="1">
       <c r="A64" s="60" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B64" s="60" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C64" s="69" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D64" s="73" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E64" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F64" s="60" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G64" s="67"/>
       <c r="H64" s="60" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="I64" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J64" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K64" s="67"/>
       <c r="L64" s="60" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="M64" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N64" s="67"/>
       <c r="O64" s="60" t="s">
@@ -15880,7 +15883,7 @@
         <v>68</v>
       </c>
       <c r="U64" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V64" s="60" t="s">
         <v>81</v>
@@ -15890,34 +15893,34 @@
       </c>
       <c r="X64" s="67"/>
       <c r="Y64" s="65" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="Z64" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="65" ht="46.5" hidden="1">
       <c r="A65" s="60" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B65" s="60" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C65" s="69" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D65" s="73" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E65" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F65" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G65" s="67"/>
       <c r="H65" s="60" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="I65" s="60" t="s">
         <v>78</v>
@@ -15927,7 +15930,7 @@
       </c>
       <c r="K65" s="67"/>
       <c r="L65" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M65" s="60" t="s">
         <v>150</v>
@@ -15963,44 +15966,44 @@
         <v>151</v>
       </c>
       <c r="Z65" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="66" ht="62" hidden="1">
       <c r="A66" s="60" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B66" s="60" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C66" s="69" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D66" s="73" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E66" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F66" s="60" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G66" s="67"/>
       <c r="H66" s="60" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="I66" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J66" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K66" s="67"/>
       <c r="L66" s="60" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="M66" s="60" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="N66" s="67"/>
       <c r="O66" s="60" t="s">
@@ -16022,44 +16025,44 @@
         <v>68</v>
       </c>
       <c r="U66" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V66" s="60" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="W66" s="60" t="s">
         <v>69</v>
       </c>
       <c r="X66" s="67"/>
       <c r="Y66" s="65" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="Z66" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="67" ht="62" hidden="1">
       <c r="A67" s="60" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B67" s="60" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C67" s="69" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D67" s="73" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E67" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F67" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G67" s="67"/>
       <c r="H67" s="60" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="I67" s="60" t="s">
         <v>78</v>
@@ -16069,7 +16072,7 @@
       </c>
       <c r="K67" s="67"/>
       <c r="L67" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M67" s="60" t="s">
         <v>150</v>
@@ -16095,7 +16098,7 @@
       </c>
       <c r="U67" s="60"/>
       <c r="V67" s="60" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="W67" s="60" t="s">
         <v>69</v>
@@ -16105,31 +16108,31 @@
         <v>151</v>
       </c>
       <c r="Z67" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="68" ht="93" hidden="1">
       <c r="A68" s="60" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B68" s="60" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C68" s="69" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D68" s="73" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E68" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F68" s="60" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="G68" s="67"/>
       <c r="H68" s="60" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="I68" s="60" t="s">
         <v>78</v>
@@ -16139,10 +16142,10 @@
       </c>
       <c r="K68" s="67"/>
       <c r="L68" s="60" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="M68" s="60" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="N68" s="67"/>
       <c r="O68" s="60" t="s">
@@ -16172,44 +16175,44 @@
       </c>
       <c r="X68" s="67"/>
       <c r="Y68" s="98" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="Z68" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="69" ht="62" hidden="1">
       <c r="A69" s="60" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B69" s="60" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C69" s="69" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D69" s="73" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E69" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F69" s="60" t="s">
         <v>154</v>
       </c>
       <c r="G69" s="67"/>
       <c r="H69" s="60" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="I69" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J69" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K69" s="67"/>
       <c r="L69" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M69" s="60" t="s">
         <v>150</v>
@@ -16234,7 +16237,7 @@
         <v>68</v>
       </c>
       <c r="U69" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V69" s="60" t="s">
         <v>81</v>
@@ -16247,44 +16250,44 @@
         <v>151</v>
       </c>
       <c r="Z69" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="70" ht="162.5" hidden="1" customHeight="1">
       <c r="A70" s="60" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B70" s="60" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C70" s="69" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D70" s="73" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E70" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F70" s="60" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="G70" s="67"/>
       <c r="H70" s="60" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="I70" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J70" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K70" s="67"/>
       <c r="L70" s="60" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="M70" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N70" s="67"/>
       <c r="O70" s="60" t="s">
@@ -16306,7 +16309,7 @@
         <v>68</v>
       </c>
       <c r="U70" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V70" s="60" t="s">
         <v>81</v>
@@ -16316,34 +16319,34 @@
       </c>
       <c r="X70" s="67"/>
       <c r="Y70" s="65" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="Z70" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="71" ht="108.5" hidden="1">
       <c r="A71" s="60" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B71" s="60" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="C71" s="69" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D71" s="73" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E71" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F71" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G71" s="67"/>
       <c r="H71" s="60" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="I71" s="60" t="s">
         <v>78</v>
@@ -16353,7 +16356,7 @@
       </c>
       <c r="K71" s="67"/>
       <c r="L71" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M71" s="60" t="s">
         <v>150</v>
@@ -16389,41 +16392,41 @@
         <v>151</v>
       </c>
       <c r="Z71" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="72" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A72" s="60" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B72" s="60" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C72" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D72" s="73" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E72" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F72" s="60" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G72" s="67"/>
       <c r="H72" s="60" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="I72" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J72" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K72" s="67"/>
       <c r="L72" s="60" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="M72" s="60"/>
       <c r="N72" s="67"/>
@@ -16446,7 +16449,7 @@
         <v>141</v>
       </c>
       <c r="U72" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V72" s="60" t="s">
         <v>69</v>
@@ -16456,34 +16459,34 @@
       </c>
       <c r="X72" s="67"/>
       <c r="Y72" s="65" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="Z72" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="73" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A73" s="60" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B73" s="60" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C73" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D73" s="73" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E73" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F73" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G73" s="67"/>
       <c r="H73" s="60" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="I73" s="60" t="s">
         <v>165</v>
@@ -16493,7 +16496,7 @@
       </c>
       <c r="K73" s="67"/>
       <c r="L73" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M73" s="60" t="s">
         <v>150</v>
@@ -16529,44 +16532,44 @@
         <v>151</v>
       </c>
       <c r="Z73" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="74" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A74" s="60" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B74" s="60" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="C74" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D74" s="73" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E74" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F74" s="60" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G74" s="67"/>
       <c r="H74" s="60" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="I74" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J74" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K74" s="67"/>
       <c r="L74" s="60" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="M74" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N74" s="67"/>
       <c r="O74" s="60" t="s">
@@ -16588,7 +16591,7 @@
         <v>68</v>
       </c>
       <c r="U74" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V74" s="60" t="s">
         <v>81</v>
@@ -16598,34 +16601,34 @@
       </c>
       <c r="X74" s="67"/>
       <c r="Y74" s="98" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="Z74" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="75" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A75" s="60" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B75" s="60" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C75" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D75" s="73" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E75" s="73" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F75" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G75" s="67"/>
       <c r="H75" s="60" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="I75" s="60" t="s">
         <v>78</v>
@@ -16635,7 +16638,7 @@
       </c>
       <c r="K75" s="67"/>
       <c r="L75" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M75" s="60" t="s">
         <v>150</v>
@@ -16671,44 +16674,44 @@
         <v>151</v>
       </c>
       <c r="Z75" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="76" ht="93" hidden="1">
       <c r="A76" s="60" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B76" s="60" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C76" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D76" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E76" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F76" s="60" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G76" s="67"/>
       <c r="H76" s="60" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="I76" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J76" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K76" s="67"/>
       <c r="L76" s="60" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="M76" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N76" s="67"/>
       <c r="O76" s="60" t="s">
@@ -16730,7 +16733,7 @@
         <v>68</v>
       </c>
       <c r="U76" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V76" s="60" t="s">
         <v>69</v>
@@ -16740,34 +16743,34 @@
       </c>
       <c r="X76" s="67"/>
       <c r="Y76" s="65" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="Z76" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="77" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A77" s="60" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B77" s="60" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C77" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D77" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E77" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F77" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G77" s="67"/>
       <c r="H77" s="60" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="I77" s="60" t="s">
         <v>78</v>
@@ -16777,7 +16780,7 @@
       </c>
       <c r="K77" s="67"/>
       <c r="L77" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M77" s="60" t="s">
         <v>150</v>
@@ -16813,44 +16816,44 @@
         <v>151</v>
       </c>
       <c r="Z77" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="78" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A78" s="60" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B78" s="60" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C78" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D78" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E78" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F78" s="60" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="G78" s="67"/>
       <c r="H78" s="60" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="I78" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J78" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K78" s="67"/>
       <c r="L78" s="60" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="M78" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N78" s="67"/>
       <c r="O78" s="60" t="s">
@@ -16872,7 +16875,7 @@
         <v>68</v>
       </c>
       <c r="U78" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V78" s="60" t="s">
         <v>69</v>
@@ -16882,34 +16885,34 @@
       </c>
       <c r="X78" s="67"/>
       <c r="Y78" s="65" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="Z78" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="79" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A79" s="60" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B79" s="60" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C79" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D79" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E79" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F79" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G79" s="67"/>
       <c r="H79" s="60" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="I79" s="60" t="s">
         <v>78</v>
@@ -16919,7 +16922,7 @@
       </c>
       <c r="K79" s="67"/>
       <c r="L79" s="60" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="M79" s="60" t="s">
         <v>150</v>
@@ -16955,31 +16958,31 @@
         <v>151</v>
       </c>
       <c r="Z79" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="80" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A80" s="60" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B80" s="60" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C80" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D80" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E80" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F80" s="60" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G80" s="67"/>
       <c r="H80" s="61" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="I80" s="61" t="s">
         <v>78</v>
@@ -16989,10 +16992,10 @@
       </c>
       <c r="K80" s="67"/>
       <c r="L80" s="60" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="M80" s="60" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N80" s="67"/>
       <c r="O80" s="60" t="s">
@@ -17014,7 +17017,7 @@
         <v>68</v>
       </c>
       <c r="U80" s="60" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="V80" s="60" t="s">
         <v>81</v>
@@ -17024,47 +17027,47 @@
       </c>
       <c r="X80" s="67"/>
       <c r="Y80" s="65" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="Z80" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="81" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A81" s="60" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B81" s="60" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C81" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D81" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E81" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F81" s="60" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G81" s="67"/>
       <c r="H81" s="60" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="I81" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J81" s="60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K81" s="67"/>
       <c r="L81" s="60" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="M81" s="60" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="N81" s="67"/>
       <c r="O81" s="60" t="s">
@@ -17086,7 +17089,7 @@
         <v>68</v>
       </c>
       <c r="U81" s="60" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="V81" s="60" t="s">
         <v>81</v>
@@ -17096,34 +17099,34 @@
       </c>
       <c r="X81" s="67"/>
       <c r="Y81" s="65" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="Z81" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="82" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A82" s="60" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B82" s="60" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C82" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D82" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E82" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F82" s="60" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="G82" s="67"/>
       <c r="H82" s="61" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="I82" s="61" t="s">
         <v>65</v>
@@ -17134,7 +17137,7 @@
       <c r="K82" s="67"/>
       <c r="L82" s="60"/>
       <c r="M82" s="61" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="N82" s="67"/>
       <c r="O82" s="60" t="s">
@@ -17165,31 +17168,31 @@
       <c r="X82" s="67"/>
       <c r="Y82" s="65"/>
       <c r="Z82" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="83" ht="62" hidden="1">
       <c r="A83" s="60" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B83" s="60" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C83" s="69" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D83" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E83" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F83" s="60" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="G83" s="67"/>
       <c r="H83" s="60" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="I83" s="60" t="s">
         <v>65</v>
@@ -17199,10 +17202,10 @@
       </c>
       <c r="K83" s="67"/>
       <c r="L83" s="60" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="M83" s="60" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="N83" s="67"/>
       <c r="O83" s="60" t="s">
@@ -17232,47 +17235,47 @@
       </c>
       <c r="X83" s="67"/>
       <c r="Y83" s="65" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="Z83" s="60" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="84" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A84" s="60" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B84" s="60" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C84" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D84" s="73" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E84" s="73" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F84" s="60" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G84" s="67"/>
       <c r="H84" s="60" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I84" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J84" s="60" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K84" s="67"/>
       <c r="L84" s="60" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="M84" s="60" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="N84" s="67"/>
       <c r="O84" s="60" t="s">
@@ -17302,34 +17305,34 @@
       </c>
       <c r="X84" s="67"/>
       <c r="Y84" s="65" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="Z84" s="60" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="85" ht="50.149999999999999" customHeight="1">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="85" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A85" s="111" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B85" s="60" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C85" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D85" s="73" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E85" s="73" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F85" s="60" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="G85" s="67"/>
       <c r="H85" s="60" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="I85" s="60" t="s">
         <v>78</v>
@@ -17339,7 +17342,7 @@
       </c>
       <c r="K85" s="67"/>
       <c r="L85" s="60" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="M85" s="60"/>
       <c r="N85" s="67"/>
@@ -17370,47 +17373,47 @@
       </c>
       <c r="X85" s="67"/>
       <c r="Y85" s="65" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="Z85" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="86" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="86" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A86" s="111" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B86" s="60" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C86" s="69" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D86" s="73" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E86" s="73" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F86" s="60" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="G86" s="67"/>
       <c r="H86" s="60" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="I86" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J86" s="60" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="K86" s="67"/>
       <c r="L86" s="60" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="M86" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N86" s="67"/>
       <c r="O86" s="60" t="s">
@@ -17432,7 +17435,7 @@
         <v>68</v>
       </c>
       <c r="U86" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V86" s="60" t="s">
         <v>81</v>
@@ -17442,40 +17445,40 @@
       </c>
       <c r="X86" s="67"/>
       <c r="Y86" s="65" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="Z86" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="87" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="87" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A87" s="111" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B87" s="60" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C87" s="69" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D87" s="73" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E87" s="73" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F87" s="60" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="G87" s="67"/>
       <c r="H87" s="60" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I87" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J87" s="60" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K87" s="67"/>
       <c r="L87" s="60"/>
@@ -17508,47 +17511,47 @@
       </c>
       <c r="X87" s="67"/>
       <c r="Y87" s="65" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="Z87" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="88" ht="46.5">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="88" ht="46.5" hidden="1">
       <c r="A88" s="111" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B88" s="60" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C88" s="69" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D88" s="73" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E88" s="73" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F88" s="60" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="G88" s="67"/>
       <c r="H88" s="60" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="I88" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J88" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K88" s="67"/>
       <c r="L88" s="60" t="s">
-        <v>615</v>
-      </c>
-      <c r="M88" s="112" t="s">
         <v>616</v>
+      </c>
+      <c r="M88" s="60" t="s">
+        <v>617</v>
       </c>
       <c r="N88" s="67"/>
       <c r="O88" s="60" t="s">
@@ -17570,7 +17573,7 @@
         <v>68</v>
       </c>
       <c r="U88" s="60" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="V88" s="60" t="s">
         <v>81</v>
@@ -17580,34 +17583,34 @@
       </c>
       <c r="X88" s="67"/>
       <c r="Y88" s="65" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="Z88" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="89" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="89" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A89" s="111" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B89" s="60" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C89" s="69" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D89" s="73" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E89" s="73" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F89" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G89" s="67"/>
       <c r="H89" s="60" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="I89" s="60" t="s">
         <v>78</v>
@@ -17617,7 +17620,7 @@
       </c>
       <c r="K89" s="67"/>
       <c r="L89" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M89" s="60" t="s">
         <v>150</v>
@@ -17653,42 +17656,42 @@
         <v>151</v>
       </c>
       <c r="Z89" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="90" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="90" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A90" s="111" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B90" s="60" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C90" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D90" s="73" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E90" s="73" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F90" s="60" t="s">
         <v>75</v>
       </c>
       <c r="G90" s="67"/>
       <c r="H90" s="60" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="I90" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J90" s="60" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K90" s="67"/>
       <c r="L90" s="60"/>
       <c r="M90" s="60" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="N90" s="67"/>
       <c r="O90" s="60" t="s">
@@ -17709,7 +17712,7 @@
       <c r="T90" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="U90" s="113"/>
+      <c r="U90" s="112"/>
       <c r="V90" s="60" t="s">
         <v>69</v>
       </c>
@@ -17718,45 +17721,45 @@
       </c>
       <c r="X90" s="67"/>
       <c r="Y90" s="65" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="Z90" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="91" ht="68.5" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="91" ht="68.5" hidden="1" customHeight="1">
       <c r="A91" s="111" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B91" s="60" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C91" s="69" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D91" s="73" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E91" s="73" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F91" s="60" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G91" s="67"/>
       <c r="H91" s="60" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="I91" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J91" s="60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K91" s="67"/>
       <c r="L91" s="60"/>
       <c r="M91" s="61" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="N91" s="67"/>
       <c r="O91" s="60" t="s">
@@ -17778,7 +17781,7 @@
         <v>141</v>
       </c>
       <c r="U91" s="60" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="V91" s="60" t="s">
         <v>69</v>
@@ -17788,47 +17791,47 @@
       </c>
       <c r="X91" s="67"/>
       <c r="Y91" s="98" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="Z91" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="92" ht="46.5">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="92" ht="46.5" hidden="1">
       <c r="A92" s="97" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B92" s="60" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C92" s="69" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D92" s="73" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E92" s="73" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F92" s="60" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G92" s="67"/>
       <c r="H92" s="60" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="I92" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J92" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K92" s="67"/>
       <c r="L92" s="60" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="M92" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N92" s="67"/>
       <c r="O92" s="60" t="s">
@@ -17850,7 +17853,7 @@
         <v>141</v>
       </c>
       <c r="U92" s="60" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="V92" s="60" t="s">
         <v>81</v>
@@ -17860,34 +17863,34 @@
       </c>
       <c r="X92" s="67"/>
       <c r="Y92" s="98" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="Z92" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="93" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="93" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A93" s="97" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B93" s="60" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C93" s="69" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D93" s="73" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E93" s="73" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F93" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G93" s="67"/>
       <c r="H93" s="60" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="I93" s="60" t="s">
         <v>165</v>
@@ -17897,7 +17900,7 @@
       </c>
       <c r="K93" s="67"/>
       <c r="L93" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M93" s="60" t="s">
         <v>150</v>
@@ -17933,44 +17936,44 @@
         <v>151</v>
       </c>
       <c r="Z93" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="94" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="94" ht="62" hidden="1">
       <c r="A94" s="97" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B94" s="60" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C94" s="69" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D94" s="73" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E94" s="73" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F94" s="60" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="G94" s="67"/>
       <c r="H94" s="60" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="I94" s="60" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="J94" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K94" s="67"/>
       <c r="L94" s="60" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="M94" s="61" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="N94" s="67"/>
       <c r="O94" s="60" t="s">
@@ -17992,7 +17995,7 @@
         <v>141</v>
       </c>
       <c r="U94" s="60" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="V94" s="60" t="s">
         <v>69</v>
@@ -18002,34 +18005,34 @@
       </c>
       <c r="X94" s="67"/>
       <c r="Y94" s="98" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="Z94" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="95" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="95" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A95" s="97" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B95" s="60" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C95" s="69" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D95" s="73" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E95" s="73" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F95" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G95" s="67"/>
       <c r="H95" s="60" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="I95" s="60" t="s">
         <v>165</v>
@@ -18039,7 +18042,7 @@
       </c>
       <c r="K95" s="67"/>
       <c r="L95" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M95" s="60" t="s">
         <v>150</v>
@@ -18075,42 +18078,42 @@
         <v>151</v>
       </c>
       <c r="Z95" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="96" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="96" ht="62" hidden="1">
       <c r="A96" s="97" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B96" s="60" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C96" s="69" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D96" s="73" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E96" s="73" t="s">
         <v>75</v>
       </c>
       <c r="F96" s="60" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="G96" s="67"/>
       <c r="H96" s="60" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="I96" s="69" t="s">
         <v>165</v>
       </c>
       <c r="J96" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K96" s="67"/>
       <c r="L96" s="60"/>
       <c r="M96" s="60" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="N96" s="67"/>
       <c r="O96" s="60" t="s">
@@ -18132,7 +18135,7 @@
         <v>141</v>
       </c>
       <c r="U96" s="60" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="V96" s="60" t="s">
         <v>81</v>
@@ -18142,24 +18145,24 @@
       </c>
       <c r="X96" s="67"/>
       <c r="Y96" s="98" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="Z96" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="97" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="97" ht="62" hidden="1">
       <c r="A97" s="97" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B97" s="97" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C97" s="69" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D97" s="73" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E97" s="73" t="s">
         <v>75</v>
@@ -18169,7 +18172,7 @@
       </c>
       <c r="G97" s="67"/>
       <c r="H97" s="60" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="I97" s="60" t="s">
         <v>165</v>
@@ -18180,7 +18183,7 @@
       <c r="K97" s="67"/>
       <c r="L97" s="60"/>
       <c r="M97" s="60" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="N97" s="67"/>
       <c r="O97" s="60" t="s">
@@ -18201,7 +18204,7 @@
       <c r="T97" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="U97" s="114"/>
+      <c r="U97" s="113"/>
       <c r="V97" s="60" t="s">
         <v>81</v>
       </c>
@@ -18213,42 +18216,42 @@
         <v>151</v>
       </c>
       <c r="Z97" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="98" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="98" ht="62" hidden="1">
       <c r="A98" s="60" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B98" s="60" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C98" s="69" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D98" s="73" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E98" s="73" t="s">
         <v>75</v>
       </c>
       <c r="F98" s="60" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="G98" s="67"/>
       <c r="H98" s="60" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="I98" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J98" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K98" s="67"/>
       <c r="L98" s="60"/>
       <c r="M98" s="60" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="N98" s="67"/>
       <c r="O98" s="60" t="s">
@@ -18270,34 +18273,34 @@
         <v>141</v>
       </c>
       <c r="U98" s="60" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="V98" s="60" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="W98" s="60" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="X98" s="67"/>
       <c r="Y98" s="98" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="Z98" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="99" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="99" ht="62" hidden="1">
       <c r="A99" s="60" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B99" s="60" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C99" s="69" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D99" s="73" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E99" s="73" t="s">
         <v>75</v>
@@ -18307,7 +18310,7 @@
       </c>
       <c r="G99" s="67"/>
       <c r="H99" s="60" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="I99" s="60" t="s">
         <v>165</v>
@@ -18318,7 +18321,7 @@
       <c r="K99" s="67"/>
       <c r="L99" s="60"/>
       <c r="M99" s="60" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="N99" s="67"/>
       <c r="O99" s="60" t="s">
@@ -18351,31 +18354,31 @@
         <v>151</v>
       </c>
       <c r="Z99" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="100" ht="77.5">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="100" ht="77.5" hidden="1">
       <c r="A100" s="97" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B100" s="60" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C100" s="69" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D100" s="73" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E100" s="73" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F100" s="60" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="G100" s="67"/>
       <c r="H100" s="60" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="I100" s="60" t="s">
         <v>165</v>
@@ -18385,7 +18388,7 @@
       </c>
       <c r="K100" s="67"/>
       <c r="L100" s="60" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="M100" s="60"/>
       <c r="N100" s="67"/>
@@ -18416,34 +18419,34 @@
       </c>
       <c r="X100" s="67"/>
       <c r="Y100" s="65" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="Z100" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="101" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="101" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A101" s="97" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B101" s="60" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C101" s="69" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D101" s="73" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E101" s="73" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F101" s="60" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="G101" s="67"/>
       <c r="H101" s="60" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="I101" s="60" t="s">
         <v>165</v>
@@ -18482,34 +18485,34 @@
       </c>
       <c r="X101" s="67"/>
       <c r="Y101" s="65" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="Z101" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="102" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="102" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A102" s="97" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B102" s="60" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C102" s="69" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D102" s="73" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E102" s="73" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F102" s="60" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="G102" s="67"/>
       <c r="H102" s="60" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="I102" s="60" t="s">
         <v>165</v>
@@ -18548,34 +18551,34 @@
       </c>
       <c r="X102" s="67"/>
       <c r="Y102" s="65" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="Z102" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="103" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="103" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A103" s="97" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B103" s="60" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C103" s="69" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D103" s="73" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E103" s="73" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F103" s="60" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="G103" s="67"/>
       <c r="H103" s="60" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="I103" s="60" t="s">
         <v>165</v>
@@ -18614,47 +18617,47 @@
       </c>
       <c r="X103" s="67"/>
       <c r="Y103" s="65" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="Z103" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="104" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="104" ht="62" hidden="1">
       <c r="A104" s="97" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B104" s="60" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C104" s="69" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="D104" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E104" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F104" s="60" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="G104" s="67"/>
       <c r="H104" s="60" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="I104" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J104" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K104" s="67"/>
       <c r="L104" s="60" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="M104" s="60" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="N104" s="67"/>
       <c r="O104" s="60" t="s">
@@ -18676,7 +18679,7 @@
         <v>68</v>
       </c>
       <c r="U104" s="60" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="V104" s="60" t="s">
         <v>69</v>
@@ -18686,34 +18689,34 @@
       </c>
       <c r="X104" s="67"/>
       <c r="Y104" s="65" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="Z104" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="105" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="105" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A105" s="97" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B105" s="60" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C105" s="69" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="D105" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E105" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F105" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G105" s="67"/>
       <c r="H105" s="60" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="I105" s="60" t="s">
         <v>78</v>
@@ -18723,7 +18726,7 @@
       </c>
       <c r="K105" s="67"/>
       <c r="L105" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M105" s="60" t="s">
         <v>150</v>
@@ -18759,31 +18762,31 @@
         <v>151</v>
       </c>
       <c r="Z105" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="106" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="106" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A106" s="97" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B106" s="60" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C106" s="69" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="D106" s="73" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E106" s="73" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F106" s="60" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G106" s="67"/>
       <c r="H106" s="60" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="I106" s="60" t="s">
         <v>78</v>
@@ -18793,10 +18796,10 @@
       </c>
       <c r="K106" s="67"/>
       <c r="L106" s="60" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="M106" s="60" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N106" s="67"/>
       <c r="O106" s="60" t="s">
@@ -18818,7 +18821,7 @@
         <v>68</v>
       </c>
       <c r="U106" s="60" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="V106" s="60" t="s">
         <v>69</v>
@@ -18828,47 +18831,47 @@
       </c>
       <c r="X106" s="67"/>
       <c r="Y106" s="65" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="Z106" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="107" ht="62">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="107" ht="62" hidden="1">
       <c r="A107" s="97" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B107" s="60" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C107" s="69" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="D107" s="73" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E107" s="73" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F107" s="60" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="G107" s="67"/>
       <c r="H107" s="60" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="I107" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J107" s="60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K107" s="67"/>
       <c r="L107" s="60" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="M107" s="60" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="N107" s="67"/>
       <c r="O107" s="60" t="s">
@@ -18890,7 +18893,7 @@
         <v>68</v>
       </c>
       <c r="U107" s="60" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="V107" s="60" t="s">
         <v>81</v>
@@ -18900,45 +18903,45 @@
       </c>
       <c r="X107" s="67"/>
       <c r="Y107" s="65" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="Z107" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="108" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="108" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A108" s="97" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B108" s="60" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C108" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D108" s="73" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E108" s="73" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F108" s="60" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G108" s="67"/>
       <c r="H108" s="60" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="I108" s="60" t="s">
         <v>78</v>
       </c>
       <c r="J108" s="60" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K108" s="67"/>
       <c r="L108" s="60"/>
       <c r="M108" s="60" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="N108" s="67"/>
       <c r="O108" s="60" t="s">
@@ -18968,45 +18971,45 @@
       </c>
       <c r="X108" s="67"/>
       <c r="Y108" s="65" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="Z108" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="109" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="109" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A109" s="97" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B109" s="60" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C109" s="69" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D109" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E109" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F109" s="60" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="G109" s="67"/>
       <c r="H109" s="60" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="I109" s="60" t="s">
         <v>65</v>
       </c>
       <c r="J109" s="60" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="K109" s="67"/>
       <c r="L109" s="60"/>
       <c r="M109" s="60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N109" s="67"/>
       <c r="O109" s="60" t="s">
@@ -19028,7 +19031,7 @@
         <v>141</v>
       </c>
       <c r="U109" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V109" s="60" t="s">
         <v>69</v>
@@ -19038,34 +19041,34 @@
       </c>
       <c r="X109" s="67"/>
       <c r="Y109" s="65" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="Z109" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="110" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="110" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A110" s="97" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B110" s="60" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C110" s="69" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D110" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E110" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F110" s="60" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="G110" s="67"/>
       <c r="H110" s="60" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="I110" s="60" t="s">
         <v>65</v>
@@ -19104,45 +19107,45 @@
       </c>
       <c r="X110" s="67"/>
       <c r="Y110" s="65" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="Z110" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="111" ht="46.5">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="111" ht="46.5" hidden="1">
       <c r="A111" s="97" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B111" s="60" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C111" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D111" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E111" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F111" s="60" t="s">
         <v>75</v>
       </c>
       <c r="G111" s="67"/>
       <c r="H111" s="60" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="I111" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J111" s="60" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="K111" s="67"/>
       <c r="L111" s="60"/>
       <c r="M111" s="60" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="N111" s="67"/>
       <c r="O111" s="60" t="s">
@@ -19163,7 +19166,7 @@
       <c r="T111" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="U111" s="113"/>
+      <c r="U111" s="112"/>
       <c r="V111" s="60" t="s">
         <v>69</v>
       </c>
@@ -19172,45 +19175,45 @@
       </c>
       <c r="X111" s="67"/>
       <c r="Y111" s="65" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="Z111" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="112" ht="93">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="112" ht="93" hidden="1">
       <c r="A112" s="97" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B112" s="60" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C112" s="69" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D112" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E112" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F112" s="60" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="G112" s="67"/>
       <c r="H112" s="60" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="I112" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J112" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K112" s="67"/>
       <c r="L112" s="60"/>
       <c r="M112" s="61" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N112" s="67"/>
       <c r="O112" s="60" t="s">
@@ -19232,7 +19235,7 @@
         <v>17</v>
       </c>
       <c r="U112" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V112" s="60" t="s">
         <v>69</v>
@@ -19242,34 +19245,34 @@
       </c>
       <c r="X112" s="67"/>
       <c r="Y112" s="65" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="Z112" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="113" ht="46.5">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="113" ht="46.5" hidden="1">
       <c r="A113" s="97" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B113" s="60" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C113" s="69" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D113" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E113" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F113" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G113" s="67"/>
       <c r="H113" s="60" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="I113" s="60" t="s">
         <v>165</v>
@@ -19279,7 +19282,7 @@
       </c>
       <c r="K113" s="67"/>
       <c r="L113" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M113" s="60" t="s">
         <v>150</v>
@@ -19315,42 +19318,42 @@
         <v>151</v>
       </c>
       <c r="Z113" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="114" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="114" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A114" s="97" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B114" s="60" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C114" s="69" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="D114" s="73" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E114" s="73" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F114" s="60" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="G114" s="67"/>
       <c r="H114" s="60" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="I114" s="60" t="s">
         <v>165</v>
       </c>
       <c r="J114" s="60" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K114" s="67"/>
       <c r="L114" s="60"/>
       <c r="M114" s="61" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="N114" s="67"/>
       <c r="O114" s="60" t="s">
@@ -19372,7 +19375,7 @@
         <v>17</v>
       </c>
       <c r="U114" s="60" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="V114" s="60" t="s">
         <v>69</v>
@@ -19382,34 +19385,34 @@
       </c>
       <c r="X114" s="67"/>
       <c r="Y114" s="65" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="Z114" s="60" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="115" ht="50.149999999999999" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="115" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A115" s="97" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B115" s="60" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C115" s="60" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="D115" s="70" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E115" s="70" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F115" s="60" t="s">
         <v>146</v>
       </c>
       <c r="G115" s="67"/>
       <c r="H115" s="60" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="I115" s="60" t="s">
         <v>165</v>
@@ -19419,7 +19422,7 @@
       </c>
       <c r="K115" s="67"/>
       <c r="L115" s="60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="M115" s="60" t="s">
         <v>150</v>
@@ -19455,7 +19458,7 @@
         <v>151</v>
       </c>
       <c r="Z115" s="60" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="116" ht="15" hidden="1" customHeight="1"/>
@@ -19463,7 +19466,7 @@
   <autoFilter ref="Z1:Z116">
     <filterColumn colId="0">
       <filters>
-        <filter val="line"/>
+        <filter val="party"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
fix: architectural view, ref: better naming
</commit_message>
<xml_diff>
--- a/docs/official/EInvoice_Data_Dictionary.xlsx
+++ b/docs/official/EInvoice_Data_Dictionary.xlsx
@@ -3058,8 +3058,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="0" tint="0"/>
+        <bgColor theme="0" tint="0"/>
       </patternFill>
     </fill>
   </fills>
@@ -12844,7 +12844,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="21" ht="50.149999999999999" customHeight="1">
+    <row r="21" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A21" s="93" t="s">
         <v>212</v>
       </c>
@@ -12914,7 +12914,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="22" ht="50.149999999999999" customHeight="1">
+    <row r="22" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A22" s="97" t="s">
         <v>223</v>
       </c>
@@ -12984,7 +12984,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="23" ht="50.149999999999999" customHeight="1">
+    <row r="23" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A23" s="60" t="s">
         <v>232</v>
       </c>
@@ -13050,7 +13050,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="24" ht="50.149999999999999" customHeight="1">
+    <row r="24" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A24" s="60" t="s">
         <v>236</v>
       </c>
@@ -13118,7 +13118,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="25" ht="50.149999999999999" customHeight="1">
+    <row r="25" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A25" s="97" t="s">
         <v>241</v>
       </c>
@@ -13188,7 +13188,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="26" ht="50.149999999999999" customHeight="1">
+    <row r="26" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A26" s="60" t="s">
         <v>247</v>
       </c>
@@ -13258,7 +13258,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="27" ht="50.149999999999999" customHeight="1">
+    <row r="27" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A27" s="97" t="s">
         <v>252</v>
       </c>
@@ -13330,7 +13330,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="28" s="99" customFormat="1" ht="50.149999999999999" customHeight="1">
+    <row r="28" s="99" customFormat="1" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A28" s="97" t="s">
         <v>259</v>
       </c>
@@ -13398,7 +13398,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="29" ht="50.149999999999999" customHeight="1">
+    <row r="29" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A29" s="61" t="s">
         <v>264</v>
       </c>
@@ -13468,7 +13468,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="30" ht="50.149999999999999" customHeight="1">
+    <row r="30" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A30" s="60" t="s">
         <v>269</v>
       </c>
@@ -13538,7 +13538,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="31" ht="129" customHeight="1">
+    <row r="31" ht="129" hidden="1" customHeight="1">
       <c r="A31" s="100" t="s">
         <v>275</v>
       </c>
@@ -13608,7 +13608,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="32" ht="50" customHeight="1">
+    <row r="32" ht="50" hidden="1" customHeight="1">
       <c r="A32" s="60" t="s">
         <v>283</v>
       </c>
@@ -13676,7 +13676,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="33" ht="50.149999999999999" customHeight="1">
+    <row r="33" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A33" s="97" t="s">
         <v>289</v>
       </c>
@@ -13749,7 +13749,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="34" ht="50.149999999999999" customHeight="1">
+    <row r="34" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A34" s="97" t="s">
         <v>223</v>
       </c>
@@ -13819,7 +13819,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="35" ht="50.149999999999999" customHeight="1">
+    <row r="35" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A35" s="97" t="s">
         <v>232</v>
       </c>
@@ -13885,7 +13885,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="36" ht="50.149999999999999" customHeight="1">
+    <row r="36" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A36" s="97" t="s">
         <v>310</v>
       </c>
@@ -13953,7 +13953,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="37" ht="50.149999999999999" customHeight="1">
+    <row r="37" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A37" s="97" t="s">
         <v>241</v>
       </c>
@@ -14019,7 +14019,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="38" ht="50.149999999999999" customHeight="1">
+    <row r="38" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A38" s="97" t="s">
         <v>247</v>
       </c>
@@ -14089,7 +14089,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="39" ht="50.149999999999999" customHeight="1">
+    <row r="39" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A39" s="97" t="s">
         <v>321</v>
       </c>
@@ -14157,7 +14157,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="40" ht="50.149999999999999" customHeight="1">
+    <row r="40" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A40" s="97" t="s">
         <v>259</v>
       </c>
@@ -14223,7 +14223,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="41" ht="50.149999999999999" customHeight="1">
+    <row r="41" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A41" s="97" t="s">
         <v>264</v>
       </c>
@@ -14291,7 +14291,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="42" ht="50.149999999999999" customHeight="1">
+    <row r="42" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A42" s="97" t="s">
         <v>269</v>
       </c>
@@ -14361,7 +14361,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="43" ht="105">
+    <row r="43" ht="105" hidden="1">
       <c r="A43" s="102" t="s">
         <v>275</v>
       </c>
@@ -14429,7 +14429,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="44" ht="50.149999999999999" customHeight="1">
+    <row r="44" ht="50.149999999999999" hidden="1" customHeight="1">
       <c r="A44" s="97" t="s">
         <v>345</v>
       </c>
@@ -17311,7 +17311,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="85" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="85" ht="50.149999999999999" customHeight="1">
       <c r="A85" s="111" t="s">
         <v>587</v>
       </c>
@@ -17379,7 +17379,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="86" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="86" ht="50.149999999999999" customHeight="1">
       <c r="A86" s="111" t="s">
         <v>596</v>
       </c>
@@ -17451,7 +17451,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="87" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="87" ht="50.149999999999999" customHeight="1">
       <c r="A87" s="111" t="s">
         <v>605</v>
       </c>
@@ -17517,7 +17517,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="88" ht="46.5" hidden="1">
+    <row r="88" ht="46.5">
       <c r="A88" s="111" t="s">
         <v>610</v>
       </c>
@@ -17589,7 +17589,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="89" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="89" ht="50.149999999999999" customHeight="1">
       <c r="A89" s="111" t="s">
         <v>619</v>
       </c>
@@ -17659,7 +17659,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="90" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="90" ht="50.149999999999999" customHeight="1">
       <c r="A90" s="111" t="s">
         <v>621</v>
       </c>
@@ -17727,7 +17727,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="91" ht="68.5" hidden="1" customHeight="1">
+    <row r="91" ht="68.5" customHeight="1">
       <c r="A91" s="111" t="s">
         <v>625</v>
       </c>
@@ -17797,7 +17797,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="92" ht="46.5" hidden="1">
+    <row r="92" ht="46.5">
       <c r="A92" s="97" t="s">
         <v>632</v>
       </c>
@@ -17869,7 +17869,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="93" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="93" ht="50.149999999999999" customHeight="1">
       <c r="A93" s="97" t="s">
         <v>430</v>
       </c>
@@ -17939,7 +17939,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="94" ht="62" hidden="1">
+    <row r="94" ht="62">
       <c r="A94" s="97" t="s">
         <v>639</v>
       </c>
@@ -18011,7 +18011,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="95" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="95" ht="50.149999999999999" customHeight="1">
       <c r="A95" s="97" t="s">
         <v>442</v>
       </c>
@@ -18081,7 +18081,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="96" ht="62" hidden="1">
+    <row r="96" ht="62">
       <c r="A96" s="97" t="s">
         <v>645</v>
       </c>
@@ -18151,7 +18151,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="97" ht="62" hidden="1">
+    <row r="97" ht="62">
       <c r="A97" s="97" t="s">
         <v>654</v>
       </c>
@@ -18219,7 +18219,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="98" ht="62" hidden="1">
+    <row r="98" ht="62">
       <c r="A98" s="60" t="s">
         <v>657</v>
       </c>
@@ -18289,7 +18289,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="99" ht="62" hidden="1">
+    <row r="99" ht="62">
       <c r="A99" s="60" t="s">
         <v>664</v>
       </c>
@@ -18357,7 +18357,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="100" ht="77.5" hidden="1">
+    <row r="100" ht="77.5">
       <c r="A100" s="97" t="s">
         <v>666</v>
       </c>
@@ -18425,7 +18425,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="101" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="101" ht="50.149999999999999" customHeight="1">
       <c r="A101" s="97" t="s">
         <v>674</v>
       </c>
@@ -18491,7 +18491,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="102" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="102" ht="50.149999999999999" customHeight="1">
       <c r="A102" s="97" t="s">
         <v>681</v>
       </c>
@@ -18557,7 +18557,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="103" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="103" ht="50.149999999999999" customHeight="1">
       <c r="A103" s="97" t="s">
         <v>686</v>
       </c>
@@ -18623,7 +18623,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="104" ht="62" hidden="1">
+    <row r="104" ht="62">
       <c r="A104" s="97" t="s">
         <v>691</v>
       </c>
@@ -18695,7 +18695,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="105" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="105" ht="50.149999999999999" customHeight="1">
       <c r="A105" s="97" t="s">
         <v>702</v>
       </c>
@@ -18765,7 +18765,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="106" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="106" ht="50.149999999999999" customHeight="1">
       <c r="A106" s="97" t="s">
         <v>704</v>
       </c>
@@ -18837,7 +18837,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="107" ht="62" hidden="1">
+    <row r="107" ht="62">
       <c r="A107" s="97" t="s">
         <v>712</v>
       </c>
@@ -18909,7 +18909,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="108" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="108" ht="50.149999999999999" customHeight="1">
       <c r="A108" s="97" t="s">
         <v>460</v>
       </c>
@@ -18977,7 +18977,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="109" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="109" ht="50.149999999999999" customHeight="1">
       <c r="A109" s="97" t="s">
         <v>720</v>
       </c>
@@ -19047,7 +19047,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="110" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="110" ht="50.149999999999999" customHeight="1">
       <c r="A110" s="97" t="s">
         <v>724</v>
       </c>
@@ -19113,7 +19113,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="111" ht="46.5" hidden="1">
+    <row r="111" ht="46.5">
       <c r="A111" s="97" t="s">
         <v>727</v>
       </c>
@@ -19181,7 +19181,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="112" ht="93" hidden="1">
+    <row r="112" ht="93">
       <c r="A112" s="97" t="s">
         <v>732</v>
       </c>
@@ -19251,7 +19251,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="113" ht="46.5" hidden="1">
+    <row r="113" ht="46.5">
       <c r="A113" s="97" t="s">
         <v>737</v>
       </c>
@@ -19321,7 +19321,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="114" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="114" ht="50.149999999999999" customHeight="1">
       <c r="A114" s="97" t="s">
         <v>739</v>
       </c>
@@ -19391,7 +19391,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="115" ht="50.149999999999999" hidden="1" customHeight="1">
+    <row r="115" ht="50.149999999999999" customHeight="1">
       <c r="A115" s="97" t="s">
         <v>745</v>
       </c>
@@ -19466,7 +19466,7 @@
   <autoFilter ref="Z1:Z116">
     <filterColumn colId="0">
       <filters>
-        <filter val="party"/>
+        <filter val="line"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
lines validation 50% complete
</commit_message>
<xml_diff>
--- a/docs/official/EInvoice_Data_Dictionary.xlsx
+++ b/docs/official/EInvoice_Data_Dictionary.xlsx
@@ -3058,8 +3058,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="0"/>
-        <bgColor theme="0" tint="0"/>
+        <fgColor indexed="5"/>
+        <bgColor indexed="5"/>
       </patternFill>
     </fill>
   </fills>
@@ -17798,7 +17798,7 @@
       </c>
     </row>
     <row r="92" ht="46.5">
-      <c r="A92" s="97" t="s">
+      <c r="A92" s="111" t="s">
         <v>632</v>
       </c>
       <c r="B92" s="60" t="s">
@@ -17870,7 +17870,7 @@
       </c>
     </row>
     <row r="93" ht="50.149999999999999" customHeight="1">
-      <c r="A93" s="97" t="s">
+      <c r="A93" s="111" t="s">
         <v>430</v>
       </c>
       <c r="B93" s="60" t="s">
@@ -18426,7 +18426,7 @@
       </c>
     </row>
     <row r="101" ht="50.149999999999999" customHeight="1">
-      <c r="A101" s="97" t="s">
+      <c r="A101" s="111" t="s">
         <v>674</v>
       </c>
       <c r="B101" s="60" t="s">
@@ -18492,7 +18492,7 @@
       </c>
     </row>
     <row r="102" ht="50.149999999999999" customHeight="1">
-      <c r="A102" s="97" t="s">
+      <c r="A102" s="111" t="s">
         <v>681</v>
       </c>
       <c r="B102" s="60" t="s">
@@ -18558,7 +18558,7 @@
       </c>
     </row>
     <row r="103" ht="50.149999999999999" customHeight="1">
-      <c r="A103" s="97" t="s">
+      <c r="A103" s="111" t="s">
         <v>686</v>
       </c>
       <c r="B103" s="60" t="s">
@@ -19048,7 +19048,7 @@
       </c>
     </row>
     <row r="110" ht="50.149999999999999" customHeight="1">
-      <c r="A110" s="97" t="s">
+      <c r="A110" s="111" t="s">
         <v>724</v>
       </c>
       <c r="B110" s="60" t="s">

</xml_diff>